<commit_message>
feat(masterdata): 판치기 타수 상한 stroke_limit=10 — 골프식
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#PanchigiConfig.xlsx
+++ b/table/Datas/#PanchigiConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,11 @@
           <t>contact_max</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>stroke_limit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -569,6 +574,11 @@
           <t>int</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -651,6 +661,11 @@
       <c r="O4" t="inlineStr">
         <is>
           <t>contact_max</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>stroke_limit</t>
         </is>
       </c>
     </row>
@@ -696,6 +711,9 @@
       </c>
       <c r="O5" t="n">
         <v>4</v>
+      </c>
+      <c r="P5" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(masterdata): 판치기 match_turn_limit·drop_out_limit 삭제 — 골프식엔 탈락·공용 턴 한도가 없다
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#PanchigiConfig.xlsx
+++ b/table/Datas/#PanchigiConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,45 +454,35 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>match_turn_limit</t>
+          <t>force_multiplier</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>drop_out_limit</t>
+          <t>horizontal_force_multiplier</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>force_multiplier</t>
+          <t>influence_radius</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>horizontal_force_multiplier</t>
+          <t>coverage_samples</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>influence_radius</t>
+          <t>hold_time_max</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>coverage_samples</t>
+          <t>contact_max</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
-        <is>
-          <t>hold_time_max</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>contact_max</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
         <is>
           <t>stroke_limit</t>
         </is>
@@ -536,45 +526,35 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>int</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -625,45 +605,35 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>match_turn_limit</t>
+          <t>force_multiplier</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>drop_out_limit</t>
+          <t>horizontal_force_multiplier</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>force_multiplier</t>
+          <t>influence_radius</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>horizontal_force_multiplier</t>
+          <t>coverage_samples</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>influence_radius</t>
+          <t>hold_time_max</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>coverage_samples</t>
+          <t>contact_max</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
-        <is>
-          <t>hold_time_max</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>contact_max</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
         <is>
           <t>stroke_limit</t>
         </is>
@@ -689,30 +659,24 @@
         <v>20</v>
       </c>
       <c r="H5" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>0.4</v>
       </c>
       <c r="K5" t="n">
-        <v>2.5</v>
+        <v>13</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="n">
-        <v>4</v>
-      </c>
-      <c r="P5" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(masterdata): 판치기 볼링 — frame_count=5, 모드 설명
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#PanchigiConfig.xlsx
+++ b/table/Datas/#PanchigiConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,11 @@
           <t>stroke_limit</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>frame_count</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +564,11 @@
           <t>int</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -636,6 +646,11 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>stroke_limit</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>frame_count</t>
         </is>
       </c>
     </row>
@@ -678,6 +693,9 @@
       </c>
       <c r="N5" t="n">
         <v>10</v>
+      </c>
+      <c r="O5" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(masterdata): 판치기 stroke_limit 삭제 — 골프식 잔재
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#PanchigiConfig.xlsx
+++ b/table/Datas/#PanchigiConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,11 +484,6 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>stroke_limit</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
           <t>frame_count</t>
         </is>
       </c>
@@ -564,11 +559,6 @@
           <t>int</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -644,11 +634,6 @@
         </is>
       </c>
       <c r="N4" t="inlineStr">
-        <is>
-          <t>stroke_limit</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
         <is>
           <t>frame_count</t>
         </is>
@@ -692,9 +677,6 @@
         <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="O5" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>